<commit_message>
feat: complete capital allocation analysis
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -49,321 +49,321 @@
     <t>capital_allocation_label</t>
   </si>
   <si>
+    <t>ABB</t>
+  </si>
+  <si>
+    <t>ADANIENSOL</t>
+  </si>
+  <si>
+    <t>ADANIENT</t>
+  </si>
+  <si>
+    <t>ADANIGREEN</t>
+  </si>
+  <si>
+    <t>ADANIPORTS</t>
+  </si>
+  <si>
+    <t>ADANIPOWER</t>
+  </si>
+  <si>
+    <t>AMBUJACEM</t>
+  </si>
+  <si>
+    <t>APOLLOHOSP</t>
+  </si>
+  <si>
+    <t>ASIANPAINT</t>
+  </si>
+  <si>
+    <t>ATGL</t>
+  </si>
+  <si>
+    <t>AXISBANK</t>
+  </si>
+  <si>
+    <t>BAJAJ-AUTO</t>
+  </si>
+  <si>
+    <t>BAJAJFINSV</t>
+  </si>
+  <si>
+    <t>BAJAJHLDNG</t>
+  </si>
+  <si>
+    <t>BAJFINANCE</t>
+  </si>
+  <si>
+    <t>BANKBARODA</t>
+  </si>
+  <si>
+    <t>BEL</t>
+  </si>
+  <si>
+    <t>BHARTIARTL</t>
+  </si>
+  <si>
+    <t>BHEL</t>
+  </si>
+  <si>
+    <t>BOSCHLTD</t>
+  </si>
+  <si>
+    <t>BPCL</t>
+  </si>
+  <si>
+    <t>BRITANNIA</t>
+  </si>
+  <si>
+    <t>CANBK</t>
+  </si>
+  <si>
+    <t>CHOLAFIN</t>
+  </si>
+  <si>
+    <t>CIPLA</t>
+  </si>
+  <si>
+    <t>COALINDIA</t>
+  </si>
+  <si>
+    <t>DABUR</t>
+  </si>
+  <si>
+    <t>DIVISLAB</t>
+  </si>
+  <si>
+    <t>DLF</t>
+  </si>
+  <si>
+    <t>DMART</t>
+  </si>
+  <si>
+    <t>DRREDDY</t>
+  </si>
+  <si>
+    <t>EICHERMOT</t>
+  </si>
+  <si>
+    <t>GAIL</t>
+  </si>
+  <si>
+    <t>GODREJCP</t>
+  </si>
+  <si>
+    <t>GRASIM</t>
+  </si>
+  <si>
+    <t>HAL</t>
+  </si>
+  <si>
+    <t>HAVELLS</t>
+  </si>
+  <si>
+    <t>HCLTECH</t>
+  </si>
+  <si>
+    <t>HDFCBANK</t>
+  </si>
+  <si>
+    <t>HDFCLIFE</t>
+  </si>
+  <si>
     <t>HEROMOTOCO</t>
   </si>
   <si>
-    <t>HDFCLIFE</t>
+    <t>HINDALCO</t>
+  </si>
+  <si>
+    <t>HINDUNILVR</t>
+  </si>
+  <si>
+    <t>ICICIBANK</t>
+  </si>
+  <si>
+    <t>ICICIGI</t>
+  </si>
+  <si>
+    <t>ICICIPRULI</t>
+  </si>
+  <si>
+    <t>INDIGO</t>
+  </si>
+  <si>
+    <t>INDUSINDBK</t>
+  </si>
+  <si>
+    <t>INFY</t>
+  </si>
+  <si>
+    <t>IOC</t>
+  </si>
+  <si>
+    <t>IRCTC</t>
+  </si>
+  <si>
+    <t>IRFC</t>
+  </si>
+  <si>
+    <t>ITC</t>
+  </si>
+  <si>
+    <t>JINDALSTEL</t>
+  </si>
+  <si>
+    <t>JIOFIN</t>
+  </si>
+  <si>
+    <t>JSWENERGY</t>
+  </si>
+  <si>
+    <t>JSWSTEEL</t>
+  </si>
+  <si>
+    <t>KOTAKBANK</t>
+  </si>
+  <si>
+    <t>LICI</t>
+  </si>
+  <si>
+    <t>LODHA</t>
+  </si>
+  <si>
+    <t>LT</t>
+  </si>
+  <si>
+    <t>LTIM</t>
+  </si>
+  <si>
+    <t>M&amp;M</t>
+  </si>
+  <si>
+    <t>MARUTI</t>
+  </si>
+  <si>
+    <t>MOTHERSON</t>
+  </si>
+  <si>
+    <t>NAUKRI</t>
+  </si>
+  <si>
+    <t>NESTLEIND</t>
+  </si>
+  <si>
+    <t>NHPC</t>
+  </si>
+  <si>
+    <t>NTPC</t>
+  </si>
+  <si>
+    <t>ONGC</t>
+  </si>
+  <si>
+    <t>PFC</t>
+  </si>
+  <si>
+    <t>PIDILITIND</t>
+  </si>
+  <si>
+    <t>PNB</t>
+  </si>
+  <si>
+    <t>POWERGRID</t>
+  </si>
+  <si>
+    <t>RECLTD</t>
+  </si>
+  <si>
+    <t>RELIANCE</t>
+  </si>
+  <si>
+    <t>SBILIFE</t>
+  </si>
+  <si>
+    <t>SBIN</t>
   </si>
   <si>
     <t>SHREECEM</t>
   </si>
   <si>
-    <t>HAL</t>
-  </si>
-  <si>
-    <t>HAVELLS</t>
-  </si>
-  <si>
-    <t>DIVISLAB</t>
+    <t>SHRIRAMFIN</t>
+  </si>
+  <si>
+    <t>SIEMENS</t>
   </si>
   <si>
     <t>SUNPHARMA</t>
   </si>
   <si>
-    <t>DABUR</t>
-  </si>
-  <si>
-    <t>GAIL</t>
-  </si>
-  <si>
-    <t>EICHERMOT</t>
-  </si>
-  <si>
-    <t>HINDALCO</t>
-  </si>
-  <si>
-    <t>SHRIRAMFIN</t>
-  </si>
-  <si>
-    <t>INDUSINDBK</t>
-  </si>
-  <si>
-    <t>RELIANCE</t>
-  </si>
-  <si>
-    <t>INDIGO</t>
-  </si>
-  <si>
-    <t>RECLTD</t>
-  </si>
-  <si>
-    <t>HCLTECH</t>
-  </si>
-  <si>
-    <t>INFY</t>
-  </si>
-  <si>
-    <t>SBIN</t>
-  </si>
-  <si>
-    <t>GRASIM</t>
-  </si>
-  <si>
-    <t>SBILIFE</t>
-  </si>
-  <si>
-    <t>NHPC</t>
-  </si>
-  <si>
-    <t>ADANIPORTS</t>
-  </si>
-  <si>
-    <t>NESTLEIND</t>
+    <t>TATACONSUM</t>
+  </si>
+  <si>
+    <t>TATAMOTORS</t>
+  </si>
+  <si>
+    <t>TATAPOWER</t>
+  </si>
+  <si>
+    <t>TATASTEEL</t>
+  </si>
+  <si>
+    <t>TCS</t>
+  </si>
+  <si>
+    <t>TECHM</t>
+  </si>
+  <si>
+    <t>TITAN</t>
   </si>
   <si>
     <t>TORNTPHARM</t>
   </si>
   <si>
-    <t>ADANIENSOL</t>
-  </si>
-  <si>
-    <t>ADANIENT</t>
-  </si>
-  <si>
-    <t>ADANIGREEN</t>
-  </si>
-  <si>
-    <t>ICICIBANK</t>
-  </si>
-  <si>
     <t>TRENT</t>
   </si>
   <si>
-    <t>NTPC</t>
-  </si>
-  <si>
-    <t>ABB</t>
-  </si>
-  <si>
-    <t>ICICIGI</t>
-  </si>
-  <si>
-    <t>HINDUNILVR</t>
-  </si>
-  <si>
-    <t>ICICIPRULI</t>
-  </si>
-  <si>
-    <t>HDFCBANK</t>
-  </si>
-  <si>
-    <t>BPCL</t>
-  </si>
-  <si>
-    <t>BOSCHLTD</t>
-  </si>
-  <si>
-    <t>TATAPOWER</t>
-  </si>
-  <si>
-    <t>BHEL</t>
-  </si>
-  <si>
-    <t>JSWSTEEL</t>
-  </si>
-  <si>
-    <t>JSWENERGY</t>
-  </si>
-  <si>
-    <t>KOTAKBANK</t>
-  </si>
-  <si>
-    <t>PNB</t>
-  </si>
-  <si>
-    <t>TATAMOTORS</t>
-  </si>
-  <si>
-    <t>TATACONSUM</t>
-  </si>
-  <si>
-    <t>DMART</t>
-  </si>
-  <si>
-    <t>CANBK</t>
-  </si>
-  <si>
-    <t>CIPLA</t>
-  </si>
-  <si>
-    <t>CHOLAFIN</t>
-  </si>
-  <si>
-    <t>JIOFIN</t>
-  </si>
-  <si>
-    <t>DLF</t>
-  </si>
-  <si>
-    <t>DRREDDY</t>
-  </si>
-  <si>
-    <t>SIEMENS</t>
-  </si>
-  <si>
-    <t>ITC</t>
-  </si>
-  <si>
-    <t>JINDALSTEL</t>
-  </si>
-  <si>
-    <t>POWERGRID</t>
-  </si>
-  <si>
-    <t>IOC</t>
-  </si>
-  <si>
-    <t>IRCTC</t>
-  </si>
-  <si>
-    <t>IRFC</t>
-  </si>
-  <si>
-    <t>COALINDIA</t>
-  </si>
-  <si>
-    <t>GODREJCP</t>
-  </si>
-  <si>
-    <t>LODHA</t>
-  </si>
-  <si>
-    <t>BHARTIARTL</t>
-  </si>
-  <si>
-    <t>TATASTEEL</t>
-  </si>
-  <si>
-    <t>LICI</t>
-  </si>
-  <si>
-    <t>BEL</t>
-  </si>
-  <si>
-    <t>BRITANNIA</t>
-  </si>
-  <si>
-    <t>BAJAJ-AUTO</t>
-  </si>
-  <si>
-    <t>TECHM</t>
-  </si>
-  <si>
-    <t>AXISBANK</t>
-  </si>
-  <si>
-    <t>TCS</t>
-  </si>
-  <si>
-    <t>PIDILITIND</t>
-  </si>
-  <si>
-    <t>PFC</t>
-  </si>
-  <si>
-    <t>LT</t>
-  </si>
-  <si>
-    <t>LTIM</t>
-  </si>
-  <si>
-    <t>BANKBARODA</t>
-  </si>
-  <si>
-    <t>BAJFINANCE</t>
-  </si>
-  <si>
-    <t>BAJAJHLDNG</t>
-  </si>
-  <si>
-    <t>TITAN</t>
-  </si>
-  <si>
-    <t>ASIANPAINT</t>
-  </si>
-  <si>
-    <t>AMBUJACEM</t>
-  </si>
-  <si>
-    <t>BAJAJFINSV</t>
-  </si>
-  <si>
-    <t>ADANIPOWER</t>
-  </si>
-  <si>
-    <t>ONGC</t>
-  </si>
-  <si>
-    <t>ATGL</t>
-  </si>
-  <si>
-    <t>APOLLOHOSP</t>
-  </si>
-  <si>
-    <t>M&amp;M</t>
-  </si>
-  <si>
-    <t>MARUTI</t>
-  </si>
-  <si>
-    <t>MOTHERSON</t>
-  </si>
-  <si>
-    <t>NAUKRI</t>
-  </si>
-  <si>
     <t>TVSMOTOR</t>
   </si>
   <si>
+    <t>Industrials</t>
+  </si>
+  <si>
+    <t>Energy</t>
+  </si>
+  <si>
+    <t>Materials</t>
+  </si>
+  <si>
+    <t>Healthcare</t>
+  </si>
+  <si>
+    <t>Financials</t>
+  </si>
+  <si>
     <t>Consumer Discretionary</t>
   </si>
   <si>
-    <t>Financials</t>
-  </si>
-  <si>
-    <t>Materials</t>
-  </si>
-  <si>
-    <t>Industrials</t>
-  </si>
-  <si>
-    <t>Healthcare</t>
+    <t>Communication Services</t>
   </si>
   <si>
     <t>Consumer Staples</t>
   </si>
   <si>
-    <t>Energy</t>
+    <t>Real Estate</t>
   </si>
   <si>
     <t>Information Technology</t>
   </si>
   <si>
-    <t>Real Estate</t>
-  </si>
-  <si>
-    <t>Communication Services</t>
-  </si>
-  <si>
     <t>High Quality</t>
   </si>
   <si>
+    <t>Accrual Risk</t>
+  </si>
+  <si>
     <t>Moderate</t>
   </si>
   <si>
-    <t>Accrual Risk</t>
-  </si>
-  <si>
     <t>Capital Intensive</t>
   </si>
   <si>
@@ -373,22 +373,22 @@
     <t>Reinvestor</t>
   </si>
   <si>
+    <t>Mixed</t>
+  </si>
+  <si>
+    <t>Liquidating Assets</t>
+  </si>
+  <si>
     <t>Growth Funded by Debt</t>
   </si>
   <si>
+    <t>Distress Signal</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
     <t>Pre-Revenue</t>
-  </si>
-  <si>
-    <t>Mixed</t>
-  </si>
-  <si>
-    <t>Unknown</t>
-  </si>
-  <si>
-    <t>Liquidating Assets</t>
-  </si>
-  <si>
-    <t>Distress Signal</t>
   </si>
 </sst>
 </file>
@@ -766,28 +766,28 @@
         <v>103</v>
       </c>
       <c r="C2">
-        <v>1.212099228421658</v>
+        <v>1.049042588613814</v>
       </c>
       <c r="D2" t="s">
         <v>113</v>
       </c>
       <c r="E2">
-        <v>4.837386541056921</v>
+        <v>7.112326893486067</v>
       </c>
       <c r="F2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G2">
-        <v>5.842708892319703</v>
+        <v>26.91956971652028</v>
       </c>
       <c r="H2">
-        <v>9.507280211341156</v>
+        <v>54.85203028217482</v>
       </c>
       <c r="I2" t="b">
         <v>0</v>
       </c>
       <c r="J2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
         <v>118</v>
@@ -801,19 +801,19 @@
         <v>104</v>
       </c>
       <c r="C3">
-        <v>5.829360645996696</v>
+        <v>4.389232826387428</v>
       </c>
       <c r="D3" t="s">
         <v>113</v>
       </c>
       <c r="E3">
-        <v>13.41518692970182</v>
+        <v>29.7645571144698</v>
       </c>
       <c r="F3" t="s">
         <v>116</v>
       </c>
       <c r="H3">
-        <v>-2.865746748422502</v>
+        <v>19.17352477674663</v>
       </c>
       <c r="I3" t="b">
         <v>0</v>
@@ -830,34 +830,31 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C4">
-        <v>1.902333713281173</v>
+        <v>3.670388196608809</v>
       </c>
       <c r="D4" t="s">
         <v>113</v>
       </c>
       <c r="E4">
-        <v>6.909994639637445</v>
+        <v>19.46360232729385</v>
       </c>
       <c r="F4" t="s">
-        <v>114</v>
-      </c>
-      <c r="G4">
-        <v>7.24045892978542</v>
+        <v>116</v>
       </c>
       <c r="H4">
-        <v>42.69588313413015</v>
+        <v>-74.31660367407929</v>
       </c>
       <c r="I4" t="b">
         <v>0</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -865,22 +862,22 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C5">
-        <v>1.963075416512269</v>
+        <v>-0.02352915575225794</v>
       </c>
       <c r="D5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E5">
-        <v>21.10529607320365</v>
+        <v>228.4164859002169</v>
       </c>
       <c r="F5" t="s">
         <v>116</v>
       </c>
       <c r="H5">
-        <v>18.60703661914042</v>
+        <v>-182.3858977862804</v>
       </c>
       <c r="I5" t="b">
         <v>0</v>
@@ -889,7 +886,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -897,31 +894,31 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C6">
-        <v>1.053161526848905</v>
+        <v>1.923293066451101</v>
       </c>
       <c r="D6" t="s">
         <v>113</v>
       </c>
       <c r="E6">
-        <v>8.703604088219473</v>
+        <v>25.33787578151324</v>
       </c>
       <c r="F6" t="s">
         <v>116</v>
       </c>
       <c r="G6">
-        <v>-13.35487386941974</v>
+        <v>37.78973446864202</v>
       </c>
       <c r="H6">
-        <v>17.80967570441255</v>
+        <v>52.92193213163128</v>
       </c>
       <c r="I6" t="b">
         <v>0</v>
       </c>
       <c r="J6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="s">
         <v>118</v>
@@ -932,25 +929,25 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C7">
-        <v>0.9293273749797603</v>
+        <v>1.3223405880104</v>
       </c>
       <c r="D7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E7">
-        <v>3.4289356277884</v>
+        <v>6.913467458441739</v>
       </c>
       <c r="F7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G7">
-        <v>29.82307104777742</v>
+        <v>30.71118060790721</v>
       </c>
       <c r="H7">
-        <v>44.8868778280543</v>
+        <v>96.83454026771999</v>
       </c>
       <c r="I7" t="b">
         <v>0</v>
@@ -959,7 +956,7 @@
         <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -967,34 +964,31 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C8">
-        <v>1.756670086239324</v>
+        <v>1.224669179404155</v>
       </c>
       <c r="D8" t="s">
         <v>113</v>
       </c>
       <c r="E8">
-        <v>1.573293193393406</v>
+        <v>26.96320868516285</v>
       </c>
       <c r="F8" t="s">
-        <v>117</v>
-      </c>
-      <c r="G8">
-        <v>43.2382586094409</v>
+        <v>116</v>
       </c>
       <c r="H8">
-        <v>87.35596865878014</v>
+        <v>-51.48437500000001</v>
       </c>
       <c r="I8" t="b">
         <v>0</v>
       </c>
       <c r="J8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1002,25 +996,25 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C9">
-        <v>1.076638358025418</v>
+        <v>3.488462128395108</v>
       </c>
       <c r="D9" t="s">
         <v>113</v>
       </c>
       <c r="E9">
-        <v>7.828119961302805</v>
+        <v>8.064431502177449</v>
       </c>
       <c r="F9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G9">
-        <v>-10.72050757546945</v>
+        <v>14.5722412524085</v>
       </c>
       <c r="H9">
-        <v>43.41666666666666</v>
+        <v>15.99832915622389</v>
       </c>
       <c r="I9" t="b">
         <v>0</v>
@@ -1037,25 +1031,25 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C10">
-        <v>0.9900484324735057</v>
+        <v>0.9321931577763529</v>
       </c>
       <c r="D10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E10">
-        <v>6.174377758429158</v>
+        <v>7.17847584166784</v>
       </c>
       <c r="F10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G10">
-        <v>13.81411233198175</v>
+        <v>18.03587045363451</v>
       </c>
       <c r="H10">
-        <v>30.45968981416794</v>
+        <v>46.88200395517469</v>
       </c>
       <c r="I10" t="b">
         <v>0</v>
@@ -1072,25 +1066,25 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C11">
-        <v>0.998535742862353</v>
+        <v>1.394198618913207</v>
       </c>
       <c r="D11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E11">
-        <v>17.13836477987421</v>
+        <v>16.80446927374302</v>
       </c>
       <c r="F11" t="s">
         <v>116</v>
       </c>
       <c r="G11">
-        <v>-0.552520013345259</v>
+        <v>-29.27279043282174</v>
       </c>
       <c r="H11">
-        <v>20.55902055902056</v>
+        <v>18.38768115942029</v>
       </c>
       <c r="I11" t="b">
         <v>0</v>
@@ -1107,34 +1101,31 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C12">
-        <v>2.765676634898685</v>
+        <v>4.970634991862178</v>
       </c>
       <c r="D12" t="s">
         <v>113</v>
       </c>
       <c r="E12">
-        <v>6.606254804085903</v>
+        <v>8.229937185125584</v>
       </c>
       <c r="F12" t="s">
-        <v>114</v>
-      </c>
-      <c r="G12">
-        <v>8.463802473474736</v>
+        <v>116</v>
       </c>
       <c r="H12">
-        <v>5.096048727159144</v>
+        <v>-38.36280736894816</v>
       </c>
       <c r="I12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1142,31 +1133,34 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C13">
-        <v>-2.612821054742972</v>
+        <v>0.7566632844852987</v>
       </c>
       <c r="D13" t="s">
         <v>115</v>
       </c>
       <c r="E13">
-        <v>0.7090249532813014</v>
+        <v>0.1604635613995989</v>
       </c>
       <c r="F13" t="s">
         <v>117</v>
       </c>
+      <c r="G13">
+        <v>23.98235048893478</v>
+      </c>
       <c r="H13">
-        <v>-298.0043713769838</v>
+        <v>73.99885909868796</v>
       </c>
       <c r="I13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" t="b">
         <v>0</v>
       </c>
       <c r="K13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1174,31 +1168,31 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C14">
-        <v>2.610541715850155</v>
+        <v>-2.993664365617242</v>
       </c>
       <c r="D14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E14">
-        <v>1.366179942292559</v>
+        <v>9.929155115870342</v>
       </c>
       <c r="F14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H14">
-        <v>-99.03617190157614</v>
+        <v>-194.7708261996772</v>
       </c>
       <c r="I14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="b">
         <v>0</v>
       </c>
       <c r="K14" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1206,28 +1200,31 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C15">
-        <v>1.614759496636935</v>
+        <v>0.3401882095534591</v>
       </c>
       <c r="D15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E15">
-        <v>12.63357288488512</v>
+        <v>27.73207990599295</v>
       </c>
       <c r="F15" t="s">
         <v>116</v>
       </c>
+      <c r="G15">
+        <v>25.86754704441738</v>
+      </c>
       <c r="H15">
-        <v>27.82003470811948</v>
+        <v>94.04609475032009</v>
       </c>
       <c r="I15" t="b">
         <v>0</v>
       </c>
       <c r="J15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" t="s">
         <v>118</v>
@@ -1238,34 +1235,31 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C16">
-        <v>-14.3446629715772</v>
+        <v>-3.758378367355445</v>
       </c>
       <c r="D16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E16">
-        <v>17.06577266922094</v>
+        <v>13.04482281888962</v>
       </c>
       <c r="F16" t="s">
         <v>116</v>
       </c>
-      <c r="G16">
-        <v>71.56520119992503</v>
-      </c>
       <c r="H16">
-        <v>17.92555113841706</v>
+        <v>-496.4966768122243</v>
       </c>
       <c r="I16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16" t="b">
         <v>0</v>
       </c>
       <c r="K16" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -1273,22 +1267,22 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C17">
-        <v>-3.856165997377703</v>
+        <v>3.473910944163455</v>
       </c>
       <c r="D17" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E17">
-        <v>3.853357745648926</v>
+        <v>1.085496583008811</v>
       </c>
       <c r="F17" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H17">
-        <v>-124.3739949460142</v>
+        <v>-17.03283084341693</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
@@ -1297,7 +1291,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -1305,25 +1299,22 @@
         <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="C18">
-        <v>1.371283984612863</v>
+        <v>1.431409743175087</v>
       </c>
       <c r="D18" t="s">
         <v>113</v>
       </c>
       <c r="E18">
-        <v>6.012027694631208</v>
+        <v>29.22834024077363</v>
       </c>
       <c r="F18" t="s">
-        <v>114</v>
-      </c>
-      <c r="G18">
-        <v>22.6161818543015</v>
+        <v>116</v>
       </c>
       <c r="H18">
-        <v>65.45995536821225</v>
+        <v>-25.04454563452781</v>
       </c>
       <c r="I18" t="b">
         <v>0</v>
@@ -1340,31 +1331,28 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C19">
-        <v>1.037696383329751</v>
+        <v>3.334066956185566</v>
       </c>
       <c r="D19" t="s">
         <v>113</v>
       </c>
       <c r="E19">
-        <v>3.314244810307802</v>
+        <v>34.06342094384659</v>
       </c>
       <c r="F19" t="s">
-        <v>114</v>
-      </c>
-      <c r="G19">
-        <v>7.201272446841034</v>
+        <v>116</v>
       </c>
       <c r="H19">
-        <v>55.22855181880576</v>
+        <v>35.51959331732489</v>
       </c>
       <c r="I19" t="b">
         <v>0</v>
       </c>
       <c r="J19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" t="s">
         <v>118</v>
@@ -1375,34 +1363,31 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C20">
-        <v>1.053882118994846</v>
+        <v>-2.210785656327544</v>
       </c>
       <c r="D20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E20">
-        <v>0.791458802474561</v>
+        <v>5.570669233666764</v>
       </c>
       <c r="F20" t="s">
-        <v>117</v>
-      </c>
-      <c r="G20">
-        <v>-9.42032384113779</v>
+        <v>115</v>
       </c>
       <c r="H20">
-        <v>-30.11095079357182</v>
+        <v>-335.0210970464135</v>
       </c>
       <c r="I20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" t="b">
         <v>0</v>
       </c>
       <c r="K20" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -1410,31 +1395,34 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C21">
-        <v>0.6128140684668629</v>
+        <v>1.073233884013101</v>
       </c>
       <c r="D21" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E21">
-        <v>17.6472384675289</v>
+        <v>1.691875411012136</v>
       </c>
       <c r="F21" t="s">
-        <v>116</v>
+        <v>117</v>
+      </c>
+      <c r="G21">
+        <v>-8.223254104876499</v>
       </c>
       <c r="H21">
-        <v>-124.408898694613</v>
+        <v>73.31742243436754</v>
       </c>
       <c r="I21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -1445,25 +1433,25 @@
         <v>104</v>
       </c>
       <c r="C22">
-        <v>15.301624757997</v>
+        <v>2.486510576648653</v>
       </c>
       <c r="D22" t="s">
         <v>113</v>
       </c>
       <c r="E22">
-        <v>23.6544231293754</v>
+        <v>2.348002490609999</v>
       </c>
       <c r="F22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H22">
-        <v>-853.2520325203253</v>
+        <v>57.65391769883399</v>
       </c>
       <c r="I22" t="b">
         <v>0</v>
       </c>
       <c r="J22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" t="s">
         <v>118</v>
@@ -1474,34 +1462,34 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C23">
-        <v>1.269192330394576</v>
+        <v>1.046539262159868</v>
       </c>
       <c r="D23" t="s">
         <v>113</v>
       </c>
       <c r="E23">
-        <v>61.96013289036545</v>
+        <v>2.844534557815016</v>
       </c>
       <c r="F23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G23">
-        <v>-18.15959230256928</v>
+        <v>58.59345160881666</v>
       </c>
       <c r="H23">
-        <v>20.17890576242979</v>
+        <v>96.30565203662772</v>
       </c>
       <c r="I23" t="b">
         <v>0</v>
       </c>
       <c r="J23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -1509,31 +1497,31 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C24">
-        <v>1.923293066451101</v>
+        <v>4.069631350415008</v>
       </c>
       <c r="D24" t="s">
         <v>113</v>
       </c>
       <c r="E24">
-        <v>25.33787578151324</v>
+        <v>1.583438141857961</v>
       </c>
       <c r="F24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G24">
-        <v>37.78973446864202</v>
+        <v>-5.337862323751841</v>
       </c>
       <c r="H24">
-        <v>52.92193213163128</v>
+        <v>28.81289819269276</v>
       </c>
       <c r="I24" t="b">
         <v>0</v>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24" t="s">
         <v>118</v>
@@ -1544,34 +1532,31 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C25">
-        <v>1.114334186875221</v>
+        <v>-6.195324924972415</v>
       </c>
       <c r="D25" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E25">
-        <v>5.070919078461917</v>
+        <v>14.89850232218337</v>
       </c>
       <c r="F25" t="s">
-        <v>114</v>
-      </c>
-      <c r="G25">
-        <v>4.320098447494725</v>
+        <v>116</v>
       </c>
       <c r="H25">
-        <v>50.54188886977465</v>
+        <v>-715.6545961002786</v>
       </c>
       <c r="I25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" t="b">
         <v>0</v>
       </c>
       <c r="K25" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -1579,25 +1564,25 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C26">
-        <v>1.831031132947694</v>
+        <v>1.412222814051014</v>
       </c>
       <c r="D26" t="s">
         <v>113</v>
       </c>
       <c r="E26">
-        <v>1.491424310216257</v>
+        <v>11.56979902227051</v>
       </c>
       <c r="F26" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G26">
-        <v>14.88463449987261</v>
+        <v>228.7503659034452</v>
       </c>
       <c r="H26">
-        <v>92.22090261282661</v>
+        <v>5.912847097469589</v>
       </c>
       <c r="I26" t="b">
         <v>0</v>
@@ -1614,22 +1599,25 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C27">
-        <v>4.389232826387428</v>
+        <v>1.021649532530456</v>
       </c>
       <c r="D27" t="s">
         <v>113</v>
       </c>
       <c r="E27">
-        <v>29.7645571144698</v>
+        <v>3.151963126387679</v>
       </c>
       <c r="F27" t="s">
-        <v>116</v>
+        <v>115</v>
+      </c>
+      <c r="G27">
+        <v>9.987217411819094</v>
       </c>
       <c r="H27">
-        <v>19.17352477674663</v>
+        <v>14.43212650500254</v>
       </c>
       <c r="I27" t="b">
         <v>0</v>
@@ -1646,22 +1634,25 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C28">
-        <v>3.670388196608809</v>
+        <v>1.076638358025418</v>
       </c>
       <c r="D28" t="s">
         <v>113</v>
       </c>
       <c r="E28">
-        <v>19.46360232729385</v>
+        <v>7.828119961302805</v>
       </c>
       <c r="F28" t="s">
-        <v>116</v>
+        <v>115</v>
+      </c>
+      <c r="G28">
+        <v>-10.72050757546945</v>
       </c>
       <c r="H28">
-        <v>-74.31660367407929</v>
+        <v>43.41666666666666</v>
       </c>
       <c r="I28" t="b">
         <v>0</v>
@@ -1670,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="K28" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -1678,31 +1669,34 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C29">
-        <v>-0.02352915575225794</v>
+        <v>0.9293273749797603</v>
       </c>
       <c r="D29" t="s">
         <v>115</v>
       </c>
       <c r="E29">
-        <v>228.4164859002169</v>
+        <v>3.4289356277884</v>
       </c>
       <c r="F29" t="s">
-        <v>116</v>
+        <v>115</v>
+      </c>
+      <c r="G29">
+        <v>29.82307104777742</v>
       </c>
       <c r="H29">
-        <v>-182.3858977862804</v>
+        <v>44.8868778280543</v>
       </c>
       <c r="I29" t="b">
         <v>0</v>
       </c>
       <c r="J29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -1710,25 +1704,25 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C30">
-        <v>3.872438044945258</v>
+        <v>0.946490479815318</v>
       </c>
       <c r="D30" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E30">
-        <v>90.7350986734873</v>
+        <v>23.79025984129454</v>
       </c>
       <c r="F30" t="s">
         <v>116</v>
       </c>
       <c r="G30">
-        <v>-7.360467011220518</v>
+        <v>-13.16733127538306</v>
       </c>
       <c r="H30">
-        <v>12.60245078344717</v>
+        <v>47.55178907721281</v>
       </c>
       <c r="I30" t="b">
         <v>0</v>
@@ -1737,7 +1731,7 @@
         <v>0</v>
       </c>
       <c r="K30" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -1745,22 +1739,22 @@
         <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C31">
-        <v>1.182341546078665</v>
+        <v>1.068669197812137</v>
       </c>
       <c r="D31" t="s">
         <v>113</v>
       </c>
       <c r="E31">
-        <v>4.105050505050505</v>
+        <v>4.859319931481227</v>
       </c>
       <c r="F31" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H31">
-        <v>42.66869609335362</v>
+        <v>6.770579639551875</v>
       </c>
       <c r="I31" t="b">
         <v>0</v>
@@ -1777,22 +1771,25 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C32">
-        <v>2.260902906732556</v>
+        <v>1.342175174052774</v>
       </c>
       <c r="D32" t="s">
         <v>113</v>
       </c>
       <c r="E32">
-        <v>18.00606159069137</v>
+        <v>14.40148513084145</v>
       </c>
       <c r="F32" t="s">
         <v>116</v>
       </c>
+      <c r="G32">
+        <v>-24.68901184980715</v>
+      </c>
       <c r="H32">
-        <v>16.7988184079602</v>
+        <v>6.416235976301525</v>
       </c>
       <c r="I32" t="b">
         <v>0</v>
@@ -1809,31 +1806,31 @@
         <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C33">
-        <v>1.049042588613814</v>
+        <v>0.998535742862353</v>
       </c>
       <c r="D33" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E33">
-        <v>7.112326893486067</v>
+        <v>17.13836477987421</v>
       </c>
       <c r="F33" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G33">
-        <v>26.91956971652028</v>
+        <v>-0.552520013345259</v>
       </c>
       <c r="H33">
-        <v>54.85203028217482</v>
+        <v>20.55902055902056</v>
       </c>
       <c r="I33" t="b">
         <v>0</v>
       </c>
       <c r="J33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="s">
         <v>118</v>
@@ -1847,22 +1844,22 @@
         <v>104</v>
       </c>
       <c r="C34">
-        <v>1.458965013017095</v>
+        <v>0.9900484324735057</v>
       </c>
       <c r="D34" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E34">
-        <v>9.37667789329819</v>
+        <v>6.174377758429158</v>
       </c>
       <c r="F34" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G34">
-        <v>32.27903093325808</v>
+        <v>13.81411233198175</v>
       </c>
       <c r="H34">
-        <v>2.71356783919598</v>
+        <v>30.45968981416794</v>
       </c>
       <c r="I34" t="b">
         <v>0</v>
@@ -1879,25 +1876,22 @@
         <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C35">
-        <v>1.156176111154535</v>
+        <v>0.1256199406068272</v>
       </c>
       <c r="D35" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E35">
-        <v>8.601525138942742</v>
+        <v>24.36861520998865</v>
       </c>
       <c r="F35" t="s">
         <v>116</v>
       </c>
-      <c r="G35">
-        <v>13.60175699592767</v>
-      </c>
       <c r="H35">
-        <v>21.47680843406652</v>
+        <v>-46.16165032127156</v>
       </c>
       <c r="I35" t="b">
         <v>0</v>
@@ -1906,7 +1900,7 @@
         <v>0</v>
       </c>
       <c r="K35" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -1914,34 +1908,31 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C36">
-        <v>1.926589234229299</v>
+        <v>0.6128140684668629</v>
       </c>
       <c r="D36" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E36">
-        <v>8.216417331989769</v>
+        <v>17.6472384675289</v>
       </c>
       <c r="F36" t="s">
         <v>116</v>
       </c>
-      <c r="G36">
-        <v>-51.26166654001434</v>
-      </c>
       <c r="H36">
-        <v>0.1139619692628289</v>
+        <v>-124.408898694613</v>
       </c>
       <c r="I36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J36" t="b">
         <v>0</v>
       </c>
       <c r="K36" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -1949,22 +1940,22 @@
         <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C37">
-        <v>0.2288453818917975</v>
+        <v>1.963075416512269</v>
       </c>
       <c r="D37" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E37">
-        <v>5.852303374945795</v>
+        <v>21.10529607320365</v>
       </c>
       <c r="F37" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H37">
-        <v>20.47635996234127</v>
+        <v>18.60703661914042</v>
       </c>
       <c r="I37" t="b">
         <v>0</v>
@@ -1973,7 +1964,7 @@
         <v>0</v>
       </c>
       <c r="K37" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -1981,28 +1972,31 @@
         <v>47</v>
       </c>
       <c r="B38" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C38">
-        <v>2.486510576648653</v>
+        <v>1.053161526848905</v>
       </c>
       <c r="D38" t="s">
         <v>113</v>
       </c>
       <c r="E38">
-        <v>2.348002490609999</v>
+        <v>8.703604088219473</v>
       </c>
       <c r="F38" t="s">
-        <v>117</v>
+        <v>116</v>
+      </c>
+      <c r="G38">
+        <v>-13.35487386941974</v>
       </c>
       <c r="H38">
-        <v>57.65391769883399</v>
+        <v>17.80967570441255</v>
       </c>
       <c r="I38" t="b">
         <v>0</v>
       </c>
       <c r="J38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K38" t="s">
         <v>118</v>
@@ -2013,34 +2007,34 @@
         <v>48</v>
       </c>
       <c r="B39" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="C39">
-        <v>1.073233884013101</v>
+        <v>1.371283984612863</v>
       </c>
       <c r="D39" t="s">
         <v>113</v>
       </c>
       <c r="E39">
-        <v>1.691875411012136</v>
+        <v>6.012027694631208</v>
       </c>
       <c r="F39" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G39">
-        <v>-8.223254104876499</v>
+        <v>22.6161818543015</v>
       </c>
       <c r="H39">
-        <v>73.31742243436754</v>
+        <v>65.45995536821225</v>
       </c>
       <c r="I39" t="b">
         <v>0</v>
       </c>
       <c r="J39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K39" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2048,25 +2042,22 @@
         <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C40">
-        <v>3.866291981206616</v>
+        <v>0.2288453818917975</v>
       </c>
       <c r="D40" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E40">
-        <v>14.69023092320461</v>
+        <v>5.852303374945795</v>
       </c>
       <c r="F40" t="s">
-        <v>116</v>
-      </c>
-      <c r="G40">
-        <v>-3.666968259247616</v>
+        <v>115</v>
       </c>
       <c r="H40">
-        <v>33.24639031206335</v>
+        <v>20.47635996234127</v>
       </c>
       <c r="I40" t="b">
         <v>0</v>
@@ -2075,7 +2066,7 @@
         <v>0</v>
       </c>
       <c r="K40" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2083,31 +2074,31 @@
         <v>50</v>
       </c>
       <c r="B41" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C41">
-        <v>-2.210785656327544</v>
+        <v>5.829360645996696</v>
       </c>
       <c r="D41" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E41">
-        <v>5.570669233666764</v>
+        <v>13.41518692970182</v>
       </c>
       <c r="F41" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H41">
-        <v>-335.0210970464135</v>
+        <v>-2.865746748422502</v>
       </c>
       <c r="I41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J41" t="b">
         <v>0</v>
       </c>
       <c r="K41" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -2115,22 +2106,25 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C42">
-        <v>2.776890673714168</v>
+        <v>1.212099228421658</v>
       </c>
       <c r="D42" t="s">
         <v>113</v>
       </c>
       <c r="E42">
-        <v>8.266573717472543</v>
+        <v>4.837386541056921</v>
       </c>
       <c r="F42" t="s">
-        <v>116</v>
+        <v>115</v>
+      </c>
+      <c r="G42">
+        <v>5.842708892319703</v>
       </c>
       <c r="H42">
-        <v>-8.484568668537131</v>
+        <v>9.507280211341156</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
@@ -2147,31 +2141,34 @@
         <v>52</v>
       </c>
       <c r="B43" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C43">
-        <v>2.627478907361001</v>
+        <v>2.765676634898685</v>
       </c>
       <c r="D43" t="s">
         <v>113</v>
       </c>
       <c r="E43">
-        <v>71.36514017064252</v>
+        <v>6.606254804085903</v>
       </c>
       <c r="F43" t="s">
-        <v>116</v>
+        <v>115</v>
+      </c>
+      <c r="G43">
+        <v>8.463802473474736</v>
       </c>
       <c r="H43">
-        <v>-36.47342995169083</v>
+        <v>5.096048727159144</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
       </c>
       <c r="J43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K43" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -2179,22 +2176,25 @@
         <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C44">
-        <v>1.475807344465532</v>
+        <v>1.156176111154535</v>
       </c>
       <c r="D44" t="s">
         <v>113</v>
       </c>
       <c r="E44">
-        <v>15.85966534487971</v>
+        <v>8.601525138942742</v>
       </c>
       <c r="F44" t="s">
         <v>116</v>
       </c>
+      <c r="G44">
+        <v>13.60175699592767</v>
+      </c>
       <c r="H44">
-        <v>14.37983507608603</v>
+        <v>21.47680843406652</v>
       </c>
       <c r="I44" t="b">
         <v>0</v>
@@ -2203,7 +2203,7 @@
         <v>0</v>
       </c>
       <c r="K44" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -2211,22 +2211,28 @@
         <v>54</v>
       </c>
       <c r="B45" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C45">
-        <v>-1.218498224295726</v>
+        <v>3.872438044945258</v>
       </c>
       <c r="D45" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E45">
-        <v>1.380827946637326</v>
+        <v>90.7350986734873</v>
       </c>
       <c r="F45" t="s">
-        <v>117</v>
+        <v>116</v>
+      </c>
+      <c r="G45">
+        <v>-7.360467011220518</v>
+      </c>
+      <c r="H45">
+        <v>12.60245078344717</v>
       </c>
       <c r="I45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J45" t="b">
         <v>0</v>
@@ -2240,28 +2246,31 @@
         <v>55</v>
       </c>
       <c r="B46" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C46">
-        <v>1.927704811215581</v>
+        <v>1.458965013017095</v>
       </c>
       <c r="D46" t="s">
         <v>113</v>
       </c>
       <c r="E46">
-        <v>5.2022250232915</v>
+        <v>9.37667789329819</v>
       </c>
       <c r="F46" t="s">
-        <v>114</v>
+        <v>116</v>
+      </c>
+      <c r="G46">
+        <v>32.27903093325808</v>
       </c>
       <c r="H46">
-        <v>75.80536800026874</v>
+        <v>2.71356783919598</v>
       </c>
       <c r="I46" t="b">
         <v>0</v>
       </c>
       <c r="J46" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K46" t="s">
         <v>118</v>
@@ -2272,25 +2281,25 @@
         <v>56</v>
       </c>
       <c r="B47" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C47">
-        <v>1.665494399678571</v>
+        <v>1.926589234229299</v>
       </c>
       <c r="D47" t="s">
         <v>113</v>
       </c>
       <c r="E47">
-        <v>12.56740760226226</v>
+        <v>8.216417331989769</v>
       </c>
       <c r="F47" t="s">
         <v>116</v>
       </c>
       <c r="G47">
-        <v>-37.04887150623013</v>
+        <v>-51.26166654001434</v>
       </c>
       <c r="H47">
-        <v>1.138353765323993</v>
+        <v>0.1139619692628289</v>
       </c>
       <c r="I47" t="b">
         <v>0</v>
@@ -2299,7 +2308,7 @@
         <v>0</v>
       </c>
       <c r="K47" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -2307,28 +2316,31 @@
         <v>57</v>
       </c>
       <c r="B48" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C48">
-        <v>1.068669197812137</v>
+        <v>-14.3446629715772</v>
       </c>
       <c r="D48" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E48">
-        <v>4.859319931481227</v>
+        <v>17.06577266922094</v>
       </c>
       <c r="F48" t="s">
-        <v>114</v>
+        <v>116</v>
+      </c>
+      <c r="G48">
+        <v>71.56520119992503</v>
       </c>
       <c r="H48">
-        <v>6.770579639551875</v>
+        <v>17.92555113841706</v>
       </c>
       <c r="I48" t="b">
         <v>0</v>
       </c>
       <c r="J48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K48" t="s">
         <v>118</v>
@@ -2339,25 +2351,22 @@
         <v>58</v>
       </c>
       <c r="B49" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C49">
-        <v>4.069631350415008</v>
+        <v>2.610541715850155</v>
       </c>
       <c r="D49" t="s">
         <v>113</v>
       </c>
       <c r="E49">
-        <v>1.583438141857961</v>
+        <v>1.366179942292559</v>
       </c>
       <c r="F49" t="s">
         <v>117</v>
       </c>
-      <c r="G49">
-        <v>-5.337862323751841</v>
-      </c>
       <c r="H49">
-        <v>28.81289819269276</v>
+        <v>-99.03617190157614</v>
       </c>
       <c r="I49" t="b">
         <v>0</v>
@@ -2366,7 +2375,7 @@
         <v>0</v>
       </c>
       <c r="K49" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -2374,31 +2383,31 @@
         <v>59</v>
       </c>
       <c r="B50" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C50">
-        <v>1.412222814051014</v>
+        <v>1.037696383329751</v>
       </c>
       <c r="D50" t="s">
         <v>113</v>
       </c>
       <c r="E50">
-        <v>11.56979902227051</v>
+        <v>3.314244810307802</v>
       </c>
       <c r="F50" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G50">
-        <v>228.7503659034452</v>
+        <v>7.201272446841034</v>
       </c>
       <c r="H50">
-        <v>5.912847097469589</v>
+        <v>55.22855181880576</v>
       </c>
       <c r="I50" t="b">
         <v>0</v>
       </c>
       <c r="J50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K50" t="s">
         <v>118</v>
@@ -2412,28 +2421,28 @@
         <v>104</v>
       </c>
       <c r="C51">
-        <v>-6.195324924972415</v>
+        <v>0.7306430873244374</v>
       </c>
       <c r="D51" t="s">
         <v>115</v>
       </c>
       <c r="E51">
-        <v>14.89850232218337</v>
+        <v>4.052800791393595</v>
       </c>
       <c r="F51" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H51">
-        <v>-715.6545961002786</v>
+        <v>52.39536789783994</v>
       </c>
       <c r="I51" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K51" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -2441,22 +2450,25 @@
         <v>61</v>
       </c>
       <c r="B52" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C52">
-        <v>32.93394633705156</v>
+        <v>0.9036900006508211</v>
       </c>
       <c r="D52" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E52">
-        <v>77.68194070080862</v>
+        <v>5.035128805620609</v>
       </c>
       <c r="F52" t="s">
-        <v>116</v>
+        <v>115</v>
+      </c>
+      <c r="G52">
+        <v>35.50477381816852</v>
       </c>
       <c r="H52">
-        <v>48.94162924951892</v>
+        <v>45.49795361527968</v>
       </c>
       <c r="I52" t="b">
         <v>0</v>
@@ -2465,7 +2477,7 @@
         <v>1</v>
       </c>
       <c r="K52" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -2473,34 +2485,31 @@
         <v>62</v>
       </c>
       <c r="B53" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C53">
-        <v>0.946490479815318</v>
+        <v>-10.79612430906241</v>
       </c>
       <c r="D53" t="s">
         <v>114</v>
       </c>
       <c r="E53">
-        <v>23.79025984129454</v>
+        <v>0.03002439482079189</v>
       </c>
       <c r="F53" t="s">
-        <v>116</v>
-      </c>
-      <c r="G53">
-        <v>-13.16733127538306</v>
+        <v>117</v>
       </c>
       <c r="H53">
-        <v>47.55178907721281</v>
+        <v>29.81933391166598</v>
       </c>
       <c r="I53" t="b">
         <v>0</v>
       </c>
       <c r="J53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K53" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -2508,34 +2517,34 @@
         <v>63</v>
       </c>
       <c r="B54" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C54">
-        <v>1.342175174052774</v>
+        <v>0.9385693291996491</v>
       </c>
       <c r="D54" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E54">
-        <v>14.40148513084145</v>
+        <v>2.205571077808822</v>
       </c>
       <c r="F54" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G54">
-        <v>-24.68901184980715</v>
+        <v>21.64259503734181</v>
       </c>
       <c r="H54">
-        <v>6.416235976301525</v>
+        <v>71.44436396904662</v>
       </c>
       <c r="I54" t="b">
         <v>0</v>
       </c>
       <c r="J54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K54" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -2543,25 +2552,22 @@
         <v>64</v>
       </c>
       <c r="B55" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C55">
-        <v>0.8407752345640682</v>
+        <v>-2.800059220273794</v>
       </c>
       <c r="D55" t="s">
         <v>114</v>
       </c>
       <c r="E55">
-        <v>2.257194244604317</v>
+        <v>16.57067958851333</v>
       </c>
       <c r="F55" t="s">
-        <v>117</v>
-      </c>
-      <c r="G55">
-        <v>53.28962129081927</v>
+        <v>116</v>
       </c>
       <c r="H55">
-        <v>37.62886597938144</v>
+        <v>-22.89747108410116</v>
       </c>
       <c r="I55" t="b">
         <v>0</v>
@@ -2570,7 +2576,7 @@
         <v>0</v>
       </c>
       <c r="K55" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="56" spans="1:11">
@@ -2578,25 +2584,22 @@
         <v>65</v>
       </c>
       <c r="B56" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C56">
-        <v>0.9385693291996491</v>
+        <v>32.93394633705156</v>
       </c>
       <c r="D56" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E56">
-        <v>2.205571077808822</v>
+        <v>77.68194070080862</v>
       </c>
       <c r="F56" t="s">
-        <v>117</v>
-      </c>
-      <c r="G56">
-        <v>21.64259503734181</v>
+        <v>116</v>
       </c>
       <c r="H56">
-        <v>71.44436396904662</v>
+        <v>48.94162924951892</v>
       </c>
       <c r="I56" t="b">
         <v>0</v>
@@ -2613,22 +2616,22 @@
         <v>66</v>
       </c>
       <c r="B57" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C57">
-        <v>-2.800059220273794</v>
+        <v>2.627478907361001</v>
       </c>
       <c r="D57" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E57">
-        <v>16.57067958851333</v>
+        <v>71.36514017064252</v>
       </c>
       <c r="F57" t="s">
         <v>116</v>
       </c>
       <c r="H57">
-        <v>-22.89747108410116</v>
+        <v>-36.47342995169083</v>
       </c>
       <c r="I57" t="b">
         <v>0</v>
@@ -2637,7 +2640,7 @@
         <v>0</v>
       </c>
       <c r="K57" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -2645,31 +2648,28 @@
         <v>67</v>
       </c>
       <c r="B58" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C58">
-        <v>2.355395296760425</v>
+        <v>2.776890673714168</v>
       </c>
       <c r="D58" t="s">
         <v>113</v>
       </c>
       <c r="E58">
-        <v>28.60633030124555</v>
+        <v>8.266573717472543</v>
       </c>
       <c r="F58" t="s">
         <v>116</v>
       </c>
-      <c r="G58">
-        <v>39.69769001638159</v>
-      </c>
       <c r="H58">
-        <v>60.70406267262592</v>
+        <v>-8.484568668537131</v>
       </c>
       <c r="I58" t="b">
         <v>0</v>
       </c>
       <c r="J58" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K58" t="s">
         <v>118</v>
@@ -2680,31 +2680,31 @@
         <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C59">
-        <v>0.7306430873244374</v>
+        <v>1.475807344465532</v>
       </c>
       <c r="D59" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E59">
-        <v>4.052800791393595</v>
+        <v>15.85966534487971</v>
       </c>
       <c r="F59" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H59">
-        <v>52.39536789783994</v>
+        <v>14.37983507608603</v>
       </c>
       <c r="I59" t="b">
         <v>0</v>
       </c>
       <c r="J59" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K59" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="60" spans="1:11">
@@ -2712,31 +2712,31 @@
         <v>69</v>
       </c>
       <c r="B60" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C60">
-        <v>0.9036900006508211</v>
+        <v>9.679944954625284</v>
       </c>
       <c r="D60" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E60">
-        <v>5.035128805620609</v>
+        <v>2.986999477520373</v>
       </c>
       <c r="F60" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G60">
-        <v>35.50477381816852</v>
+        <v>-48.21728841371581</v>
       </c>
       <c r="H60">
-        <v>45.49795361527968</v>
+        <v>2.602275847341285</v>
       </c>
       <c r="I60" t="b">
         <v>0</v>
       </c>
       <c r="J60" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K60" t="s">
         <v>118</v>
@@ -2747,31 +2747,31 @@
         <v>70</v>
       </c>
       <c r="B61" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C61">
-        <v>-10.79612430906241</v>
+        <v>13.30991666183648</v>
       </c>
       <c r="D61" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E61">
-        <v>0.03002439482079189</v>
+        <v>28.5672741372625</v>
       </c>
       <c r="F61" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H61">
-        <v>29.81933391166598</v>
+        <v>-16.32270168855535</v>
       </c>
       <c r="I61" t="b">
         <v>0</v>
       </c>
       <c r="J61" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K61" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -2779,25 +2779,22 @@
         <v>71</v>
       </c>
       <c r="B62" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C62">
-        <v>1.021649532530456</v>
+        <v>1.446423006390699</v>
       </c>
       <c r="D62" t="s">
         <v>113</v>
       </c>
       <c r="E62">
-        <v>3.151963126387679</v>
+        <v>0.9854689683555468</v>
       </c>
       <c r="F62" t="s">
-        <v>114</v>
-      </c>
-      <c r="G62">
-        <v>9.987217411819094</v>
+        <v>117</v>
       </c>
       <c r="H62">
-        <v>14.43212650500254</v>
+        <v>68.45806127574083</v>
       </c>
       <c r="I62" t="b">
         <v>0</v>
@@ -2806,7 +2803,7 @@
         <v>0</v>
       </c>
       <c r="K62" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="63" spans="1:11">
@@ -2814,22 +2811,25 @@
         <v>72</v>
       </c>
       <c r="B63" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C63">
-        <v>0.1256199406068272</v>
+        <v>1.016292459052437</v>
       </c>
       <c r="D63" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E63">
-        <v>24.36861520998865</v>
+        <v>11.03133710617451</v>
       </c>
       <c r="F63" t="s">
         <v>116</v>
       </c>
+      <c r="G63">
+        <v>22.08444037386408</v>
+      </c>
       <c r="H63">
-        <v>-46.16165032127156</v>
+        <v>27.43071864725223</v>
       </c>
       <c r="I63" t="b">
         <v>0</v>
@@ -2838,7 +2838,7 @@
         <v>0</v>
       </c>
       <c r="K63" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="64" spans="1:11">
@@ -2846,25 +2846,25 @@
         <v>73</v>
       </c>
       <c r="B64" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C64">
-        <v>13.30991666183648</v>
+        <v>3.315557726769421</v>
       </c>
       <c r="D64" t="s">
         <v>113</v>
       </c>
       <c r="E64">
-        <v>28.5672741372625</v>
+        <v>4.037302808495951</v>
       </c>
       <c r="F64" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H64">
-        <v>-16.32270168855535</v>
+        <v>-45.17515667684396</v>
       </c>
       <c r="I64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J64" t="b">
         <v>0</v>
@@ -2878,22 +2878,25 @@
         <v>74</v>
       </c>
       <c r="B65" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C65">
-        <v>3.334066956185566</v>
+        <v>1.132404458201285</v>
       </c>
       <c r="D65" t="s">
         <v>113</v>
       </c>
       <c r="E65">
-        <v>34.06342094384659</v>
+        <v>8.363997800617518</v>
       </c>
       <c r="F65" t="s">
         <v>116</v>
       </c>
+      <c r="G65">
+        <v>10.02778351575371</v>
+      </c>
       <c r="H65">
-        <v>35.51959331732489</v>
+        <v>26.50059057231827</v>
       </c>
       <c r="I65" t="b">
         <v>0</v>
@@ -2910,22 +2913,25 @@
         <v>75</v>
       </c>
       <c r="B66" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C66">
-        <v>4.441136197317481</v>
+        <v>3.099669015457905</v>
       </c>
       <c r="D66" t="s">
         <v>113</v>
       </c>
       <c r="E66">
-        <v>6.219373306395661</v>
+        <v>6.732055283102987</v>
       </c>
       <c r="F66" t="s">
-        <v>114</v>
+        <v>115</v>
+      </c>
+      <c r="G66">
+        <v>-1.428567128563307</v>
       </c>
       <c r="H66">
-        <v>27.18446601941747</v>
+        <v>9.922763355503111</v>
       </c>
       <c r="I66" t="b">
         <v>0</v>
@@ -2934,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="K66" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="67" spans="1:11">
@@ -2942,25 +2948,22 @@
         <v>76</v>
       </c>
       <c r="B67" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C67">
-        <v>9.679944954625284</v>
+        <v>-1.461538977694653</v>
       </c>
       <c r="D67" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E67">
-        <v>2.986999477520373</v>
+        <v>33.59621451104101</v>
       </c>
       <c r="F67" t="s">
-        <v>117</v>
-      </c>
-      <c r="G67">
-        <v>-48.21728841371581</v>
+        <v>116</v>
       </c>
       <c r="H67">
-        <v>2.602275847341285</v>
+        <v>-21.09704641350211</v>
       </c>
       <c r="I67" t="b">
         <v>0</v>
@@ -2969,7 +2972,7 @@
         <v>0</v>
       </c>
       <c r="K67" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="68" spans="1:11">
@@ -2977,22 +2980,25 @@
         <v>77</v>
       </c>
       <c r="B68" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C68">
-        <v>1.431409743175087</v>
+        <v>1.114334186875221</v>
       </c>
       <c r="D68" t="s">
         <v>113</v>
       </c>
       <c r="E68">
-        <v>29.22834024077363</v>
+        <v>5.070919078461917</v>
       </c>
       <c r="F68" t="s">
-        <v>116</v>
+        <v>115</v>
+      </c>
+      <c r="G68">
+        <v>4.320098447494725</v>
       </c>
       <c r="H68">
-        <v>-25.04454563452781</v>
+        <v>50.54188886977465</v>
       </c>
       <c r="I68" t="b">
         <v>0</v>
@@ -3009,34 +3015,34 @@
         <v>78</v>
       </c>
       <c r="B69" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C69">
-        <v>1.046539262159868</v>
+        <v>1.269192330394576</v>
       </c>
       <c r="D69" t="s">
         <v>113</v>
       </c>
       <c r="E69">
-        <v>2.844534557815016</v>
+        <v>61.96013289036545</v>
       </c>
       <c r="F69" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G69">
-        <v>58.59345160881666</v>
+        <v>-18.15959230256928</v>
       </c>
       <c r="H69">
-        <v>96.30565203662772</v>
+        <v>20.17890576242979</v>
       </c>
       <c r="I69" t="b">
         <v>0</v>
       </c>
       <c r="J69" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K69" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -3044,25 +3050,22 @@
         <v>79</v>
       </c>
       <c r="B70" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C70">
-        <v>0.7566632844852987</v>
+        <v>2.260902906732556</v>
       </c>
       <c r="D70" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E70">
-        <v>0.1604635613995989</v>
+        <v>18.00606159069137</v>
       </c>
       <c r="F70" t="s">
-        <v>117</v>
-      </c>
-      <c r="G70">
-        <v>23.98235048893478</v>
+        <v>116</v>
       </c>
       <c r="H70">
-        <v>73.99885909868796</v>
+        <v>16.7988184079602</v>
       </c>
       <c r="I70" t="b">
         <v>0</v>
@@ -3079,31 +3082,31 @@
         <v>80</v>
       </c>
       <c r="B71" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C71">
-        <v>1.544725287120112</v>
+        <v>2.864497231939887</v>
       </c>
       <c r="D71" t="s">
         <v>113</v>
       </c>
       <c r="E71">
-        <v>2.534810370028464</v>
+        <v>9.672537521390066</v>
       </c>
       <c r="F71" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G71">
-        <v>16.78825509724664</v>
+        <v>11.57315479777334</v>
       </c>
       <c r="H71">
-        <v>112.2503328894807</v>
+        <v>40.90047162930909</v>
       </c>
       <c r="I71" t="b">
         <v>0</v>
       </c>
       <c r="J71" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K71" t="s">
         <v>118</v>
@@ -3114,22 +3117,22 @@
         <v>81</v>
       </c>
       <c r="B72" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C72">
-        <v>4.970634991862178</v>
+        <v>-3.034796145263461</v>
       </c>
       <c r="D72" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E72">
-        <v>8.229937185125584</v>
+        <v>3.725357345805831</v>
       </c>
       <c r="F72" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H72">
-        <v>-38.36280736894816</v>
+        <v>-301.5190778303994</v>
       </c>
       <c r="I72" t="b">
         <v>1</v>
@@ -3138,7 +3141,7 @@
         <v>0</v>
       </c>
       <c r="K72" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="73" spans="1:11">
@@ -3146,34 +3149,34 @@
         <v>82</v>
       </c>
       <c r="B73" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C73">
-        <v>1.036410569304885</v>
+        <v>1.187241128670088</v>
       </c>
       <c r="D73" t="s">
         <v>113</v>
       </c>
       <c r="E73">
-        <v>2.528508507926756</v>
+        <v>14.28571428571428</v>
       </c>
       <c r="F73" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G73">
-        <v>10.77084245698778</v>
+        <v>23.53017525858574</v>
       </c>
       <c r="H73">
-        <v>78.43256190120692</v>
+        <v>35.2658788774003</v>
       </c>
       <c r="I73" t="b">
         <v>0</v>
       </c>
       <c r="J73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K73" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="74" spans="1:11">
@@ -3181,34 +3184,28 @@
         <v>83</v>
       </c>
       <c r="B74" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C74">
-        <v>1.187241128670088</v>
+        <v>-1.218498224295726</v>
       </c>
       <c r="D74" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E74">
-        <v>14.28571428571428</v>
+        <v>1.380827946637326</v>
       </c>
       <c r="F74" t="s">
-        <v>116</v>
-      </c>
-      <c r="G74">
-        <v>23.53017525858574</v>
-      </c>
-      <c r="H74">
-        <v>35.2658788774003</v>
+        <v>117</v>
       </c>
       <c r="I74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J74" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K74" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="75" spans="1:11">
@@ -3219,28 +3216,31 @@
         <v>104</v>
       </c>
       <c r="C75">
-        <v>-3.034796145263461</v>
+        <v>2.355395296760425</v>
       </c>
       <c r="D75" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E75">
-        <v>3.725357345805831</v>
+        <v>28.60633030124555</v>
       </c>
       <c r="F75" t="s">
-        <v>114</v>
+        <v>116</v>
+      </c>
+      <c r="G75">
+        <v>39.69769001638159</v>
       </c>
       <c r="H75">
-        <v>-301.5190778303994</v>
+        <v>60.70406267262592</v>
       </c>
       <c r="I75" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K75" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="76" spans="1:11">
@@ -3248,31 +3248,31 @@
         <v>85</v>
       </c>
       <c r="B76" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C76">
-        <v>1.446423006390699</v>
+        <v>-3.856165997377703</v>
       </c>
       <c r="D76" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E76">
-        <v>0.9854689683555468</v>
+        <v>3.853357745648926</v>
       </c>
       <c r="F76" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H76">
-        <v>68.45806127574083</v>
+        <v>-124.3739949460142</v>
       </c>
       <c r="I76" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J76" t="b">
         <v>0</v>
       </c>
       <c r="K76" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="77" spans="1:11">
@@ -3280,25 +3280,22 @@
         <v>86</v>
       </c>
       <c r="B77" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C77">
-        <v>1.016292459052437</v>
+        <v>1.614759496636935</v>
       </c>
       <c r="D77" t="s">
         <v>113</v>
       </c>
       <c r="E77">
-        <v>11.03133710617451</v>
+        <v>12.63357288488512</v>
       </c>
       <c r="F77" t="s">
         <v>116</v>
       </c>
-      <c r="G77">
-        <v>22.08444037386408</v>
-      </c>
       <c r="H77">
-        <v>27.43071864725223</v>
+        <v>27.82003470811948</v>
       </c>
       <c r="I77" t="b">
         <v>0</v>
@@ -3315,31 +3312,31 @@
         <v>87</v>
       </c>
       <c r="B78" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C78">
-        <v>3.473910944163455</v>
+        <v>15.301624757997</v>
       </c>
       <c r="D78" t="s">
         <v>113</v>
       </c>
       <c r="E78">
-        <v>1.085496583008811</v>
+        <v>23.6544231293754</v>
       </c>
       <c r="F78" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H78">
-        <v>-17.03283084341693</v>
+        <v>-853.2520325203253</v>
       </c>
       <c r="I78" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J78" t="b">
         <v>0</v>
       </c>
       <c r="K78" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="79" spans="1:11">
@@ -3347,31 +3344,34 @@
         <v>88</v>
       </c>
       <c r="B79" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C79">
-        <v>-3.758378367355445</v>
+        <v>1.053882118994846</v>
       </c>
       <c r="D79" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E79">
-        <v>13.04482281888962</v>
+        <v>0.791458802474561</v>
       </c>
       <c r="F79" t="s">
-        <v>116</v>
+        <v>117</v>
+      </c>
+      <c r="G79">
+        <v>-9.42032384113779</v>
       </c>
       <c r="H79">
-        <v>-496.4966768122243</v>
+        <v>-30.11095079357182</v>
       </c>
       <c r="I79" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J79" t="b">
         <v>0</v>
       </c>
       <c r="K79" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="80" spans="1:11">
@@ -3379,25 +3379,25 @@
         <v>89</v>
       </c>
       <c r="B80" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C80">
-        <v>0.3401882095534591</v>
+        <v>1.902333713281173</v>
       </c>
       <c r="D80" t="s">
+        <v>113</v>
+      </c>
+      <c r="E80">
+        <v>6.909994639637445</v>
+      </c>
+      <c r="F80" t="s">
         <v>115</v>
       </c>
-      <c r="E80">
-        <v>27.73207990599295</v>
-      </c>
-      <c r="F80" t="s">
-        <v>116</v>
-      </c>
       <c r="G80">
-        <v>25.86754704441738</v>
+        <v>7.24045892978542</v>
       </c>
       <c r="H80">
-        <v>94.04609475032009</v>
+        <v>42.69588313413015</v>
       </c>
       <c r="I80" t="b">
         <v>0</v>
@@ -3414,34 +3414,31 @@
         <v>90</v>
       </c>
       <c r="B81" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C81">
-        <v>0.9180593506856705</v>
+        <v>-2.612821054742972</v>
       </c>
       <c r="D81" t="s">
         <v>114</v>
       </c>
       <c r="E81">
-        <v>0.3699788583509513</v>
+        <v>0.7090249532813014</v>
       </c>
       <c r="F81" t="s">
         <v>117</v>
       </c>
-      <c r="G81">
-        <v>27.55515729109304</v>
-      </c>
       <c r="H81">
-        <v>28.45804988662132</v>
+        <v>-298.0043713769838</v>
       </c>
       <c r="I81" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J81" t="b">
         <v>0</v>
       </c>
       <c r="K81" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="82" spans="1:11">
@@ -3449,25 +3446,25 @@
         <v>91</v>
       </c>
       <c r="B82" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C82">
-        <v>0.9321931577763529</v>
+        <v>0.8407752345640682</v>
       </c>
       <c r="D82" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E82">
-        <v>7.17847584166784</v>
+        <v>2.257194244604317</v>
       </c>
       <c r="F82" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G82">
-        <v>18.03587045363451</v>
+        <v>53.28962129081927</v>
       </c>
       <c r="H82">
-        <v>46.88200395517469</v>
+        <v>37.62886597938144</v>
       </c>
       <c r="I82" t="b">
         <v>0</v>
@@ -3484,31 +3481,34 @@
         <v>92</v>
       </c>
       <c r="B83" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C83">
-        <v>1.224669179404155</v>
+        <v>1.756670086239324</v>
       </c>
       <c r="D83" t="s">
         <v>113</v>
       </c>
       <c r="E83">
-        <v>26.96320868516285</v>
+        <v>1.573293193393406</v>
       </c>
       <c r="F83" t="s">
-        <v>116</v>
+        <v>117</v>
+      </c>
+      <c r="G83">
+        <v>43.2382586094409</v>
       </c>
       <c r="H83">
-        <v>-51.48437500000001</v>
+        <v>87.35596865878014</v>
       </c>
       <c r="I83" t="b">
         <v>0</v>
       </c>
       <c r="J83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K83" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="84" spans="1:11">
@@ -3516,25 +3516,28 @@
         <v>93</v>
       </c>
       <c r="B84" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C84">
-        <v>-2.993664365617242</v>
+        <v>1.665494399678571</v>
       </c>
       <c r="D84" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E84">
-        <v>9.929155115870342</v>
+        <v>12.56740760226226</v>
       </c>
       <c r="F84" t="s">
         <v>116</v>
       </c>
+      <c r="G84">
+        <v>-37.04887150623013</v>
+      </c>
       <c r="H84">
-        <v>-194.7708261996772</v>
+        <v>1.138353765323993</v>
       </c>
       <c r="I84" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J84" t="b">
         <v>0</v>
@@ -3548,25 +3551,22 @@
         <v>94</v>
       </c>
       <c r="B85" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C85">
-        <v>1.3223405880104</v>
+        <v>1.927704811215581</v>
       </c>
       <c r="D85" t="s">
         <v>113</v>
       </c>
       <c r="E85">
-        <v>6.913467458441739</v>
+        <v>5.2022250232915</v>
       </c>
       <c r="F85" t="s">
-        <v>114</v>
-      </c>
-      <c r="G85">
-        <v>30.71118060790721</v>
+        <v>115</v>
       </c>
       <c r="H85">
-        <v>96.83454026771999</v>
+        <v>75.80536800026874</v>
       </c>
       <c r="I85" t="b">
         <v>0</v>
@@ -3575,7 +3575,7 @@
         <v>1</v>
       </c>
       <c r="K85" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="86" spans="1:11">
@@ -3583,25 +3583,25 @@
         <v>95</v>
       </c>
       <c r="B86" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C86">
-        <v>2.864497231939887</v>
+        <v>3.866291981206616</v>
       </c>
       <c r="D86" t="s">
         <v>113</v>
       </c>
       <c r="E86">
-        <v>9.672537521390066</v>
+        <v>14.69023092320461</v>
       </c>
       <c r="F86" t="s">
         <v>116</v>
       </c>
       <c r="G86">
-        <v>11.57315479777334</v>
+        <v>-3.666968259247616</v>
       </c>
       <c r="H86">
-        <v>40.90047162930909</v>
+        <v>33.24639031206335</v>
       </c>
       <c r="I86" t="b">
         <v>0</v>
@@ -3618,25 +3618,22 @@
         <v>96</v>
       </c>
       <c r="B87" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C87">
-        <v>1.394198618913207</v>
+        <v>4.441136197317481</v>
       </c>
       <c r="D87" t="s">
         <v>113</v>
       </c>
       <c r="E87">
-        <v>16.80446927374302</v>
+        <v>6.219373306395661</v>
       </c>
       <c r="F87" t="s">
-        <v>116</v>
-      </c>
-      <c r="G87">
-        <v>-29.27279043282174</v>
+        <v>115</v>
       </c>
       <c r="H87">
-        <v>18.38768115942029</v>
+        <v>27.18446601941747</v>
       </c>
       <c r="I87" t="b">
         <v>0</v>
@@ -3653,25 +3650,25 @@
         <v>97</v>
       </c>
       <c r="B88" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C88">
-        <v>3.488462128395108</v>
+        <v>1.036410569304885</v>
       </c>
       <c r="D88" t="s">
         <v>113</v>
       </c>
       <c r="E88">
-        <v>8.064431502177449</v>
+        <v>2.528508507926756</v>
       </c>
       <c r="F88" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G88">
-        <v>14.5722412524085</v>
+        <v>10.77084245698778</v>
       </c>
       <c r="H88">
-        <v>15.99832915622389</v>
+        <v>78.43256190120692</v>
       </c>
       <c r="I88" t="b">
         <v>0</v>
@@ -3680,7 +3677,7 @@
         <v>0</v>
       </c>
       <c r="K88" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="89" spans="1:11">
@@ -3688,31 +3685,34 @@
         <v>98</v>
       </c>
       <c r="B89" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="C89">
-        <v>3.315557726769421</v>
+        <v>1.544725287120112</v>
       </c>
       <c r="D89" t="s">
         <v>113</v>
       </c>
       <c r="E89">
-        <v>4.037302808495951</v>
+        <v>2.534810370028464</v>
       </c>
       <c r="F89" t="s">
-        <v>114</v>
+        <v>117</v>
+      </c>
+      <c r="G89">
+        <v>16.78825509724664</v>
       </c>
       <c r="H89">
-        <v>-45.17515667684396</v>
+        <v>112.2503328894807</v>
       </c>
       <c r="I89" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K89" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="90" spans="1:11">
@@ -3720,31 +3720,31 @@
         <v>99</v>
       </c>
       <c r="B90" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C90">
-        <v>1.132404458201285</v>
+        <v>0.9180593506856705</v>
       </c>
       <c r="D90" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E90">
-        <v>8.363997800617518</v>
+        <v>0.3699788583509513</v>
       </c>
       <c r="F90" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G90">
-        <v>10.02778351575371</v>
+        <v>27.55515729109304</v>
       </c>
       <c r="H90">
-        <v>26.50059057231827</v>
+        <v>28.45804988662132</v>
       </c>
       <c r="I90" t="b">
         <v>0</v>
       </c>
       <c r="J90" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K90" t="s">
         <v>118</v>
@@ -3755,34 +3755,34 @@
         <v>100</v>
       </c>
       <c r="B91" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C91">
-        <v>3.099669015457905</v>
+        <v>1.831031132947694</v>
       </c>
       <c r="D91" t="s">
         <v>113</v>
       </c>
       <c r="E91">
-        <v>6.732055283102987</v>
+        <v>1.491424310216257</v>
       </c>
       <c r="F91" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="G91">
-        <v>-1.428567128563307</v>
+        <v>14.88463449987261</v>
       </c>
       <c r="H91">
-        <v>9.922763355503111</v>
+        <v>92.22090261282661</v>
       </c>
       <c r="I91" t="b">
         <v>0</v>
       </c>
       <c r="J91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K91" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -3790,31 +3790,31 @@
         <v>101</v>
       </c>
       <c r="B92" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C92">
-        <v>-1.461538977694653</v>
+        <v>1.182341546078665</v>
       </c>
       <c r="D92" t="s">
+        <v>113</v>
+      </c>
+      <c r="E92">
+        <v>4.105050505050505</v>
+      </c>
+      <c r="F92" t="s">
         <v>115</v>
       </c>
-      <c r="E92">
-        <v>33.59621451104101</v>
-      </c>
-      <c r="F92" t="s">
-        <v>116</v>
-      </c>
       <c r="H92">
-        <v>-21.09704641350211</v>
+        <v>42.66869609335362</v>
       </c>
       <c r="I92" t="b">
         <v>0</v>
       </c>
       <c r="J92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K92" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="93" spans="1:11">
@@ -3822,13 +3822,13 @@
         <v>102</v>
       </c>
       <c r="B93" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C93">
         <v>-0.7508952449451183</v>
       </c>
       <c r="D93" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E93">
         <v>2.557159279601482</v>
@@ -3846,7 +3846,7 @@
         <v>0</v>
       </c>
       <c r="K93" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>